<commit_message>
Mistake fixup - orphacodes from tar syndrome to 1q21.1-1q21.2
</commit_message>
<xml_diff>
--- a/data/input/cnv_data.xlsx
+++ b/data/input/cnv_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\alexandra\cnv-data\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\alexandra\chapter1\cnv-data\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1CF571D-4BCC-409D-A448-5F7A5F2993DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9224E83-3390-4902-B2A6-48D22785BFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cnv_input_table" sheetId="1" r:id="rId1"/>
@@ -2351,7 +2351,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>38</v>
@@ -2378,7 +2378,7 @@
         <v>10</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="K4" s="9" t="s">
         <v>10</v>

</xml_diff>